<commit_message>
CATA-CD v2: capability-validated adaptive teacher agent + deployable change adapter
- Rebuild models/ for new main line: A2Net+DCA, distill (cache_v2/teacher_package/kd/probe), agent (signature/registry/bandit), 8 teacher backbones in thirdparty/, tools (cache gen/audit/smoke/agent), train.py

- Simplify others/ teacher repos (sam2/dinov2/dinov3/RemoteCLIP/MaRS/AnySat/UniverSat/RADIO) to LICENSE+README

- Add train_scripts/CATA-CD (teacher_adaptation + Run1); clean README; add .gitignore; extend extract_metrics/models_to_txt
</commit_message>
<xml_diff>
--- a/docs/experiment_metrics.xlsx
+++ b/docs/experiment_metrics.xlsx
@@ -188,8 +188,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ExperimentResultsTable" displayName="ExperimentResultsTable" ref="A1:AE76" headerRowCount="1">
-  <autoFilter ref="A1:AE76"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ExperimentResultsTable" displayName="ExperimentResultsTable" ref="A1:AE86" headerRowCount="1">
+  <autoFilter ref="A1:AE86"/>
   <tableColumns count="31">
     <tableColumn id="1" name="Run"/>
     <tableColumn id="2" name="Stage"/>
@@ -516,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -538,7 +538,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-09-23 08:49:08 +0800</t>
+          <t>2026-09-24 11:57:18 +0800</t>
         </is>
       </c>
     </row>
@@ -574,7 +574,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>outputs/DirectionC (DART-R) + outputs/DART-R-TS + outputs/RDT-CD + outputs/SCTC; launcher logs excluded</t>
+          <t>outputs/DirectionC (DART-R) + outputs/DART-R-TS + outputs/RDT-CD + outputs/SCTC + outputs/SAGE-CD; launcher logs excluded</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8">
@@ -596,7 +596,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>DART-R=8, DART-R-TS=4, FA-SCRD-Run1=8, RDT-CD-Run1=12, RDT-CD-Run2=11, RDT-CD-Run3=14, SAGE-CD-Run1=6, SCTC-Run1=12</t>
+          <t>DART-R=8, DART-R-TS=4, FA-SCRD-Run1=8, RDT-CD-Run1=12, RDT-CD-Run2=11, RDT-CD-Run3=14, SAGE-CD-Run1=6, SAGE-CD-Run2=10, SCTC-Run1=12</t>
         </is>
       </c>
     </row>
@@ -645,6 +645,18 @@
       <c r="B12" s="3" t="inlineStr">
         <is>
           <t>SAGE-CD-Run1 (Safe-DINO gate): G0=clean, G1=joint temporal BN, G2=full-res DINO semantic target + aux head + logit standardization + gradient budget. G2-G1 = WHU +0.46 / SYSU -0.25 → gate FAIL (SYSU), WHU-only again; but KD mechanism fixed (kd 12-15→0.6, grad budget ~25%). 40k, seed 2333 only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>SAGE-CD Run2 scope</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>SAGE-CD-Run2 (failure-type routed native-scale dual-expert distillation + symmetric context fusion): R0=clean A2Net, R1=+joint temporal BN, R2=+SCF + identity-centered decoder gate, R3=+DINO semantic (1/16) + SAM boundary (1/4) uniform, R4=+failure-type reliability routing (main method). R4-R2 (main gate, needs &gt;=+0.30 on both) = SYSU -0.44 / WHU +0.18 → FAIL. R4-R3 = SYSU +0.19 / WHU +0.02. All 10 runs completed 40000 steps, swap/deploy error 0, deploy 2.9131M / 2.7676G. 40k, seed 2333 only.</t>
         </is>
       </c>
     </row>
@@ -659,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE76"/>
+  <dimension ref="A1:AE86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2260,7 +2272,7 @@
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; joint_bn=True; teacher=True</t>
         </is>
       </c>
       <c r="G14" s="5" t="n">
@@ -2369,7 +2381,7 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; joint_bn=True; teacher=True</t>
         </is>
       </c>
       <c r="G15" s="5" t="n">
@@ -2478,7 +2490,7 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; joint_bn=False; teacher=False</t>
         </is>
       </c>
       <c r="G16" s="5" t="n">
@@ -2587,7 +2599,7 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; joint_bn=False; teacher=False</t>
         </is>
       </c>
       <c r="G17" s="5" t="n">
@@ -2696,7 +2708,7 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; joint_bn=True; teacher=False</t>
         </is>
       </c>
       <c r="G18" s="5" t="n">
@@ -2805,7 +2817,7 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; joint_bn=True; teacher=False</t>
         </is>
       </c>
       <c r="G19" s="5" t="n">
@@ -2914,7 +2926,7 @@
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; joint_bn=True; teacher=True</t>
         </is>
       </c>
       <c r="G20" s="5" t="n">
@@ -3023,7 +3035,7 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; joint_bn=True; teacher=True</t>
         </is>
       </c>
       <c r="G21" s="5" t="n">
@@ -7387,7 +7399,7 @@
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; joint_bn=False; teacher=False</t>
         </is>
       </c>
       <c r="G59" s="5" t="n">
@@ -7496,7 +7508,7 @@
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; joint_bn=False; teacher=False</t>
         </is>
       </c>
       <c r="G60" s="5" t="n">
@@ -7605,7 +7617,7 @@
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; joint_bn=True; teacher=False</t>
         </is>
       </c>
       <c r="G61" s="5" t="n">
@@ -7714,7 +7726,7 @@
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; joint_bn=True; teacher=False</t>
         </is>
       </c>
       <c r="G62" s="5" t="n">
@@ -7823,7 +7835,7 @@
       </c>
       <c r="F63" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; joint_bn=True; teacher=True</t>
         </is>
       </c>
       <c r="G63" s="5" t="n">
@@ -7932,7 +7944,7 @@
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; joint_bn=True; teacher=True</t>
         </is>
       </c>
       <c r="G64" s="5" t="n">
@@ -8016,7 +8028,7 @@
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>SCTC-Run1</t>
+          <t>SAGE-CD-Run2</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
@@ -8026,22 +8038,22 @@
       </c>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>S0</t>
+          <t>R0</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>S0_Clean_A2Net_LWGANet_L0</t>
+          <t>R0</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=none</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; dice=batch; joint_bn=False; scf=False; gate=False; teacher=False; routing=False</t>
         </is>
       </c>
       <c r="G65" s="5" t="n">
@@ -8064,9 +8076,7 @@
       <c r="L65" s="7" t="n">
         <v>0.0001</v>
       </c>
-      <c r="M65" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="M65" s="5" t="n"/>
       <c r="N65" s="5" t="inlineStr">
         <is>
           <t>batch</t>
@@ -8085,22 +8095,22 @@
         <v>2.7676</v>
       </c>
       <c r="U65" s="8" t="n">
-        <v>97.68770000000001</v>
+        <v>80.1767</v>
       </c>
       <c r="V65" s="8" t="n">
-        <v>97.8814</v>
+        <v>86.2732</v>
       </c>
       <c r="W65" s="8" t="n">
-        <v>99.45359999999999</v>
+        <v>92.3167</v>
       </c>
       <c r="X65" s="8" t="n">
-        <v>97.78449999999999</v>
+        <v>83.1133</v>
       </c>
       <c r="Y65" s="8" t="n">
-        <v>95.66500000000001</v>
+        <v>71.10590000000001</v>
       </c>
       <c r="Z65" s="8" t="n">
-        <v>97.47280000000001</v>
+        <v>78.149</v>
       </c>
       <c r="AA65" s="9" t="n"/>
       <c r="AB65" s="9" t="n">
@@ -8108,24 +8118,24 @@
       </c>
       <c r="AC65" s="5" t="inlineStr">
         <is>
-          <t>3:42:46.634404</t>
+          <t>2:54:28.038880</t>
         </is>
       </c>
       <c r="AD65" s="5" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1</t>
+          <t>outputs/SAGE-CD/Run2</t>
         </is>
       </c>
       <c r="AE65" s="6" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1/S0/CDD/train_log.txt</t>
+          <t>outputs/SAGE-CD/Run2/R0/SYSU/train_log.txt</t>
         </is>
       </c>
     </row>
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>SCTC-Run1</t>
+          <t>SAGE-CD-Run2</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr">
@@ -8135,22 +8145,22 @@
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>S0</t>
+          <t>R0</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>S0_Clean_A2Net_LWGANet_L0</t>
+          <t>R0</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=none</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; dice=batch; joint_bn=False; scf=False; gate=False; teacher=False; routing=False</t>
         </is>
       </c>
       <c r="G66" s="5" t="n">
@@ -8173,9 +8183,7 @@
       <c r="L66" s="7" t="n">
         <v>0.0001</v>
       </c>
-      <c r="M66" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="M66" s="5" t="n"/>
       <c r="N66" s="5" t="inlineStr">
         <is>
           <t>batch</t>
@@ -8194,22 +8202,22 @@
         <v>2.7676</v>
       </c>
       <c r="U66" s="8" t="n">
-        <v>89.4019</v>
+        <v>90.22409999999999</v>
       </c>
       <c r="V66" s="8" t="n">
-        <v>92.447</v>
+        <v>95.857</v>
       </c>
       <c r="W66" s="8" t="n">
-        <v>99.08799999999999</v>
+        <v>99.45739999999999</v>
       </c>
       <c r="X66" s="8" t="n">
-        <v>90.8989</v>
+        <v>92.95529999999999</v>
       </c>
       <c r="Y66" s="8" t="n">
-        <v>83.3163</v>
+        <v>86.8378</v>
       </c>
       <c r="Z66" s="8" t="n">
-        <v>90.41900000000001</v>
+        <v>92.6734</v>
       </c>
       <c r="AA66" s="9" t="n"/>
       <c r="AB66" s="9" t="n">
@@ -8217,24 +8225,24 @@
       </c>
       <c r="AC66" s="5" t="inlineStr">
         <is>
-          <t>2:47:14.389924</t>
+          <t>2:43:42.870592</t>
         </is>
       </c>
       <c r="AD66" s="5" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1</t>
+          <t>outputs/SAGE-CD/Run2</t>
         </is>
       </c>
       <c r="AE66" s="6" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1/S0/LEVIR/train_log.txt</t>
+          <t>outputs/SAGE-CD/Run2/R0/WHU/train_log.txt</t>
         </is>
       </c>
     </row>
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>SCTC-Run1</t>
+          <t>SAGE-CD-Run2</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr">
@@ -8244,12 +8252,12 @@
       </c>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>S0</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>S0_Clean_A2Net_LWGANet_L0</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -8259,7 +8267,7 @@
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=none</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; dice=batch; joint_bn=True; scf=False; gate=False; teacher=False; routing=False</t>
         </is>
       </c>
       <c r="G67" s="5" t="n">
@@ -8282,9 +8290,7 @@
       <c r="L67" s="7" t="n">
         <v>0.0001</v>
       </c>
-      <c r="M67" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="M67" s="5" t="n"/>
       <c r="N67" s="5" t="inlineStr">
         <is>
           <t>batch</t>
@@ -8303,22 +8309,22 @@
         <v>2.7676</v>
       </c>
       <c r="U67" s="8" t="n">
-        <v>81.14139999999999</v>
+        <v>79.2176</v>
       </c>
       <c r="V67" s="8" t="n">
-        <v>84.9704</v>
+        <v>86.1065</v>
       </c>
       <c r="W67" s="8" t="n">
-        <v>92.1679</v>
+        <v>92.08460000000001</v>
       </c>
       <c r="X67" s="8" t="n">
-        <v>83.01180000000001</v>
+        <v>82.51849999999999</v>
       </c>
       <c r="Y67" s="8" t="n">
-        <v>70.9573</v>
+        <v>70.2396</v>
       </c>
       <c r="Z67" s="8" t="n">
-        <v>77.92609999999999</v>
+        <v>77.41409999999999</v>
       </c>
       <c r="AA67" s="9" t="n"/>
       <c r="AB67" s="9" t="n">
@@ -8326,24 +8332,24 @@
       </c>
       <c r="AC67" s="5" t="inlineStr">
         <is>
-          <t>2:20:47.929272</t>
+          <t>2:42:50.776756</t>
         </is>
       </c>
       <c r="AD67" s="5" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1</t>
+          <t>outputs/SAGE-CD/Run2</t>
         </is>
       </c>
       <c r="AE67" s="6" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1/S0/SYSU/train_log.txt</t>
+          <t>outputs/SAGE-CD/Run2/R1/SYSU/train_log.txt</t>
         </is>
       </c>
     </row>
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>SCTC-Run1</t>
+          <t>SAGE-CD-Run2</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr">
@@ -8353,12 +8359,12 @@
       </c>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>S0</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>S0_Clean_A2Net_LWGANet_L0</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -8368,7 +8374,7 @@
       </c>
       <c r="F68" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=none</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; dice=batch; joint_bn=True; scf=False; gate=False; teacher=False; routing=False</t>
         </is>
       </c>
       <c r="G68" s="5" t="n">
@@ -8391,9 +8397,7 @@
       <c r="L68" s="7" t="n">
         <v>0.0001</v>
       </c>
-      <c r="M68" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="M68" s="5" t="n"/>
       <c r="N68" s="5" t="inlineStr">
         <is>
           <t>batch</t>
@@ -8412,22 +8416,22 @@
         <v>2.7676</v>
       </c>
       <c r="U68" s="8" t="n">
-        <v>91.9434</v>
+        <v>91.3554</v>
       </c>
       <c r="V68" s="8" t="n">
-        <v>95.20650000000001</v>
+        <v>95.5201</v>
       </c>
       <c r="W68" s="8" t="n">
-        <v>99.4967</v>
+        <v>99.48700000000001</v>
       </c>
       <c r="X68" s="8" t="n">
-        <v>93.54649999999999</v>
+        <v>93.3913</v>
       </c>
       <c r="Y68" s="8" t="n">
-        <v>87.87549999999999</v>
+        <v>87.602</v>
       </c>
       <c r="Z68" s="8" t="n">
-        <v>93.2847</v>
+        <v>93.1246</v>
       </c>
       <c r="AA68" s="9" t="n"/>
       <c r="AB68" s="9" t="n">
@@ -8435,24 +8439,24 @@
       </c>
       <c r="AC68" s="5" t="inlineStr">
         <is>
-          <t>2:43:01.630317</t>
+          <t>2:35:15.092315</t>
         </is>
       </c>
       <c r="AD68" s="5" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1</t>
+          <t>outputs/SAGE-CD/Run2</t>
         </is>
       </c>
       <c r="AE68" s="6" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1/S0/WHU/train_log.txt</t>
+          <t>outputs/SAGE-CD/Run2/R1/WHU/train_log.txt</t>
         </is>
       </c>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>SCTC-Run1</t>
+          <t>SAGE-CD-Run2</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr">
@@ -8462,22 +8466,22 @@
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>S1_FullPixel_Symmetric_Calibration</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="F69" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=symmetric</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; dice=batch; joint_bn=True; scf=True; gate=True; teacher=False; routing=False</t>
         </is>
       </c>
       <c r="G69" s="5" t="n">
@@ -8500,9 +8504,7 @@
       <c r="L69" s="7" t="n">
         <v>0.0001</v>
       </c>
-      <c r="M69" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="M69" s="5" t="n"/>
       <c r="N69" s="5" t="inlineStr">
         <is>
           <t>batch</t>
@@ -8521,22 +8523,22 @@
         <v>2.7676</v>
       </c>
       <c r="U69" s="8" t="n">
-        <v>97.39619999999999</v>
+        <v>79.08370000000001</v>
       </c>
       <c r="V69" s="8" t="n">
-        <v>97.7011</v>
+        <v>85.9074</v>
       </c>
       <c r="W69" s="8" t="n">
-        <v>99.39570000000001</v>
+        <v>92.00789999999999</v>
       </c>
       <c r="X69" s="8" t="n">
-        <v>97.5484</v>
+        <v>82.3544</v>
       </c>
       <c r="Y69" s="8" t="n">
-        <v>95.21420000000001</v>
+        <v>70.0022</v>
       </c>
       <c r="Z69" s="8" t="n">
-        <v>97.2038</v>
+        <v>77.1999</v>
       </c>
       <c r="AA69" s="9" t="n"/>
       <c r="AB69" s="9" t="n">
@@ -8544,24 +8546,24 @@
       </c>
       <c r="AC69" s="5" t="inlineStr">
         <is>
-          <t>3:19:01.505607</t>
+          <t>3:14:23.037150</t>
         </is>
       </c>
       <c r="AD69" s="5" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1</t>
+          <t>outputs/SAGE-CD/Run2</t>
         </is>
       </c>
       <c r="AE69" s="6" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1/S1/CDD/train_log.txt</t>
+          <t>outputs/SAGE-CD/Run2/R2/SYSU/train_log.txt</t>
         </is>
       </c>
     </row>
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>SCTC-Run1</t>
+          <t>SAGE-CD-Run2</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr">
@@ -8571,22 +8573,22 @@
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>S1_FullPixel_Symmetric_Calibration</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=symmetric</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; dice=batch; joint_bn=True; scf=True; gate=True; teacher=False; routing=False</t>
         </is>
       </c>
       <c r="G70" s="5" t="n">
@@ -8609,9 +8611,7 @@
       <c r="L70" s="7" t="n">
         <v>0.0001</v>
       </c>
-      <c r="M70" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="M70" s="5" t="n"/>
       <c r="N70" s="5" t="inlineStr">
         <is>
           <t>batch</t>
@@ -8630,22 +8630,22 @@
         <v>2.7676</v>
       </c>
       <c r="U70" s="8" t="n">
-        <v>89.7944</v>
+        <v>92.0291</v>
       </c>
       <c r="V70" s="8" t="n">
-        <v>92.1617</v>
+        <v>95.3805</v>
       </c>
       <c r="W70" s="8" t="n">
-        <v>99.0911</v>
+        <v>99.5069</v>
       </c>
       <c r="X70" s="8" t="n">
-        <v>90.96260000000001</v>
+        <v>93.6748</v>
       </c>
       <c r="Y70" s="8" t="n">
-        <v>83.4233</v>
+        <v>88.1022</v>
       </c>
       <c r="Z70" s="8" t="n">
-        <v>90.4842</v>
+        <v>93.41840000000001</v>
       </c>
       <c r="AA70" s="9" t="n"/>
       <c r="AB70" s="9" t="n">
@@ -8653,24 +8653,24 @@
       </c>
       <c r="AC70" s="5" t="inlineStr">
         <is>
-          <t>0:33:15.349976</t>
+          <t>3:05:47.496618</t>
         </is>
       </c>
       <c r="AD70" s="5" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1</t>
+          <t>outputs/SAGE-CD/Run2</t>
         </is>
       </c>
       <c r="AE70" s="6" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1/S1/LEVIR/train_log.txt</t>
+          <t>outputs/SAGE-CD/Run2/R2/WHU/train_log.txt</t>
         </is>
       </c>
     </row>
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>SCTC-Run1</t>
+          <t>SAGE-CD-Run2</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr">
@@ -8680,12 +8680,12 @@
       </c>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>S1_FullPixel_Symmetric_Calibration</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -8695,7 +8695,7 @@
       </c>
       <c r="F71" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=symmetric</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; dice=batch; joint_bn=True; scf=True; gate=True; teacher=True; routing=False</t>
         </is>
       </c>
       <c r="G71" s="5" t="n">
@@ -8718,9 +8718,7 @@
       <c r="L71" s="7" t="n">
         <v>0.0001</v>
       </c>
-      <c r="M71" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="M71" s="5" t="n"/>
       <c r="N71" s="5" t="inlineStr">
         <is>
           <t>batch</t>
@@ -8739,22 +8737,22 @@
         <v>2.7676</v>
       </c>
       <c r="U71" s="8" t="n">
-        <v>80.42610000000001</v>
+        <v>77.79509999999999</v>
       </c>
       <c r="V71" s="8" t="n">
-        <v>85.6097</v>
+        <v>86.0711</v>
       </c>
       <c r="W71" s="8" t="n">
-        <v>92.19580000000001</v>
+        <v>91.7945</v>
       </c>
       <c r="X71" s="8" t="n">
-        <v>82.93700000000001</v>
+        <v>81.72409999999999</v>
       </c>
       <c r="Y71" s="8" t="n">
-        <v>70.8481</v>
+        <v>69.0962</v>
       </c>
       <c r="Z71" s="8" t="n">
-        <v>77.8843</v>
+        <v>76.45110000000001</v>
       </c>
       <c r="AA71" s="9" t="n"/>
       <c r="AB71" s="9" t="n">
@@ -8762,24 +8760,24 @@
       </c>
       <c r="AC71" s="5" t="inlineStr">
         <is>
-          <t>3:32:56.072083</t>
+          <t>3:51:41.094501</t>
         </is>
       </c>
       <c r="AD71" s="5" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1</t>
+          <t>outputs/SAGE-CD/Run2</t>
         </is>
       </c>
       <c r="AE71" s="6" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1/S1/SYSU/train_log.txt</t>
+          <t>outputs/SAGE-CD/Run2/R3/SYSU/train_log.txt</t>
         </is>
       </c>
     </row>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>SCTC-Run1</t>
+          <t>SAGE-CD-Run2</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr">
@@ -8789,12 +8787,12 @@
       </c>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>S1</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>S1_FullPixel_Symmetric_Calibration</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -8804,7 +8802,7 @@
       </c>
       <c r="F72" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=symmetric</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; dice=batch; joint_bn=True; scf=True; gate=True; teacher=True; routing=False</t>
         </is>
       </c>
       <c r="G72" s="5" t="n">
@@ -8827,9 +8825,7 @@
       <c r="L72" s="7" t="n">
         <v>0.0001</v>
       </c>
-      <c r="M72" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="M72" s="5" t="n"/>
       <c r="N72" s="5" t="inlineStr">
         <is>
           <t>batch</t>
@@ -8848,22 +8844,22 @@
         <v>2.7676</v>
       </c>
       <c r="U72" s="8" t="n">
-        <v>92.1589</v>
+        <v>91.9157</v>
       </c>
       <c r="V72" s="8" t="n">
-        <v>95.1091</v>
+        <v>95.84049999999999</v>
       </c>
       <c r="W72" s="8" t="n">
-        <v>99.5009</v>
+        <v>99.521</v>
       </c>
       <c r="X72" s="8" t="n">
-        <v>93.61070000000001</v>
+        <v>93.83709999999999</v>
       </c>
       <c r="Y72" s="8" t="n">
-        <v>87.9889</v>
+        <v>88.3897</v>
       </c>
       <c r="Z72" s="8" t="n">
-        <v>93.3511</v>
+        <v>93.58800000000001</v>
       </c>
       <c r="AA72" s="9" t="n"/>
       <c r="AB72" s="9" t="n">
@@ -8871,24 +8867,24 @@
       </c>
       <c r="AC72" s="5" t="inlineStr">
         <is>
-          <t>2:40:44.864364</t>
+          <t>3:44:11.925094</t>
         </is>
       </c>
       <c r="AD72" s="5" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1</t>
+          <t>outputs/SAGE-CD/Run2</t>
         </is>
       </c>
       <c r="AE72" s="6" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1/S1/WHU/train_log.txt</t>
+          <t>outputs/SAGE-CD/Run2/R3/WHU/train_log.txt</t>
         </is>
       </c>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>SCTC-Run1</t>
+          <t>SAGE-CD-Run2</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr">
@@ -8898,22 +8894,22 @@
       </c>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>S2_SCTC_UnchangedAware_Symmetric_CrossTemporal_Calibration</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
-          <t>CDD-CD-256</t>
+          <t>SYSU-CD-256</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=sctc</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; dice=batch; joint_bn=True; scf=True; gate=True; teacher=True; routing=True</t>
         </is>
       </c>
       <c r="G73" s="5" t="n">
@@ -8936,9 +8932,7 @@
       <c r="L73" s="7" t="n">
         <v>0.0001</v>
       </c>
-      <c r="M73" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="M73" s="5" t="n"/>
       <c r="N73" s="5" t="inlineStr">
         <is>
           <t>batch</t>
@@ -8957,22 +8951,22 @@
         <v>2.7676</v>
       </c>
       <c r="U73" s="8" t="n">
-        <v>97.4438</v>
+        <v>77.655</v>
       </c>
       <c r="V73" s="8" t="n">
-        <v>97.71940000000001</v>
+        <v>86.6653</v>
       </c>
       <c r="W73" s="8" t="n">
-        <v>99.4038</v>
+        <v>91.9127</v>
       </c>
       <c r="X73" s="8" t="n">
-        <v>97.5814</v>
+        <v>81.9131</v>
       </c>
       <c r="Y73" s="8" t="n">
-        <v>95.277</v>
+        <v>69.3668</v>
       </c>
       <c r="Z73" s="8" t="n">
-        <v>97.2414</v>
+        <v>76.7252</v>
       </c>
       <c r="AA73" s="9" t="n"/>
       <c r="AB73" s="9" t="n">
@@ -8980,24 +8974,24 @@
       </c>
       <c r="AC73" s="5" t="inlineStr">
         <is>
-          <t>2:52:30.285254</t>
+          <t>3:36:32.815452</t>
         </is>
       </c>
       <c r="AD73" s="5" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1</t>
+          <t>outputs/SAGE-CD/Run2</t>
         </is>
       </c>
       <c r="AE73" s="6" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1/S2/CDD/train_log.txt</t>
+          <t>outputs/SAGE-CD/Run2/R4/SYSU/train_log.txt</t>
         </is>
       </c>
     </row>
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>SCTC-Run1</t>
+          <t>SAGE-CD-Run2</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr">
@@ -9007,22 +9001,22 @@
       </c>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>S2_SCTC_UnchangedAware_Symmetric_CrossTemporal_Calibration</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>LEVIR-CD-256</t>
+          <t>WHU-CD-256</t>
         </is>
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=sctc</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; dice=batch; joint_bn=True; scf=True; gate=True; teacher=True; routing=True</t>
         </is>
       </c>
       <c r="G74" s="5" t="n">
@@ -9045,9 +9039,7 @@
       <c r="L74" s="7" t="n">
         <v>0.0001</v>
       </c>
-      <c r="M74" s="5" t="n">
-        <v>1</v>
-      </c>
+      <c r="M74" s="5" t="n"/>
       <c r="N74" s="5" t="inlineStr">
         <is>
           <t>batch</t>
@@ -9066,22 +9058,22 @@
         <v>2.7676</v>
       </c>
       <c r="U74" s="8" t="n">
-        <v>90.1421</v>
+        <v>91.9663</v>
       </c>
       <c r="V74" s="8" t="n">
-        <v>91.4601</v>
+        <v>95.8237</v>
       </c>
       <c r="W74" s="8" t="n">
-        <v>99.069</v>
+        <v>99.5222</v>
       </c>
       <c r="X74" s="8" t="n">
-        <v>90.7963</v>
+        <v>93.8554</v>
       </c>
       <c r="Y74" s="8" t="n">
-        <v>83.14399999999999</v>
+        <v>88.42219999999999</v>
       </c>
       <c r="Z74" s="8" t="n">
-        <v>90.3061</v>
+        <v>93.60690000000001</v>
       </c>
       <c r="AA74" s="9" t="n"/>
       <c r="AB74" s="9" t="n">
@@ -9089,17 +9081,17 @@
       </c>
       <c r="AC74" s="5" t="inlineStr">
         <is>
-          <t>3:18:11.767618</t>
+          <t>3:45:05.674031</t>
         </is>
       </c>
       <c r="AD74" s="5" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1</t>
+          <t>outputs/SAGE-CD/Run2</t>
         </is>
       </c>
       <c r="AE74" s="6" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1/S2/LEVIR/train_log.txt</t>
+          <t>outputs/SAGE-CD/Run2/R4/WHU/train_log.txt</t>
         </is>
       </c>
     </row>
@@ -9116,22 +9108,22 @@
       </c>
       <c r="C75" s="5" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S0</t>
         </is>
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>S2_SCTC_UnchangedAware_Symmetric_CrossTemporal_Calibration</t>
+          <t>S0_Clean_A2Net_LWGANet_L0</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>SYSU-CD-256</t>
+          <t>CDD-CD-256</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=sctc</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=none</t>
         </is>
       </c>
       <c r="G75" s="5" t="n">
@@ -9175,22 +9167,22 @@
         <v>2.7676</v>
       </c>
       <c r="U75" s="8" t="n">
-        <v>81.00070000000001</v>
+        <v>97.68770000000001</v>
       </c>
       <c r="V75" s="8" t="n">
-        <v>84.595</v>
+        <v>97.8814</v>
       </c>
       <c r="W75" s="8" t="n">
-        <v>92.04090000000001</v>
+        <v>99.45359999999999</v>
       </c>
       <c r="X75" s="8" t="n">
-        <v>82.75879999999999</v>
+        <v>97.78449999999999</v>
       </c>
       <c r="Y75" s="8" t="n">
-        <v>70.5885</v>
+        <v>95.66500000000001</v>
       </c>
       <c r="Z75" s="8" t="n">
-        <v>77.5882</v>
+        <v>97.47280000000001</v>
       </c>
       <c r="AA75" s="9" t="n"/>
       <c r="AB75" s="9" t="n">
@@ -9198,7 +9190,7 @@
       </c>
       <c r="AC75" s="5" t="inlineStr">
         <is>
-          <t>4:06:34.060509</t>
+          <t>3:42:46.634404</t>
         </is>
       </c>
       <c r="AD75" s="5" t="inlineStr">
@@ -9208,7 +9200,7 @@
       </c>
       <c r="AE75" s="6" t="inlineStr">
         <is>
-          <t>outputs/SCTC/Run1/S2/SYSU/train_log.txt</t>
+          <t>outputs/SCTC/Run1/S0/CDD/train_log.txt</t>
         </is>
       </c>
     </row>
@@ -9225,22 +9217,22 @@
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>S2</t>
+          <t>S0</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>S2_SCTC_UnchangedAware_Symmetric_CrossTemporal_Calibration</t>
+          <t>S0_Clean_A2Net_LWGANet_L0</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>WHU-CD-256</t>
+          <t>LEVIR-CD-256</t>
         </is>
       </c>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=sctc</t>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=none</t>
         </is>
       </c>
       <c r="G76" s="5" t="n">
@@ -9284,22 +9276,22 @@
         <v>2.7676</v>
       </c>
       <c r="U76" s="8" t="n">
-        <v>92.7942</v>
+        <v>89.4019</v>
       </c>
       <c r="V76" s="8" t="n">
-        <v>95.1825</v>
+        <v>92.447</v>
       </c>
       <c r="W76" s="8" t="n">
-        <v>99.5278</v>
+        <v>99.08799999999999</v>
       </c>
       <c r="X76" s="8" t="n">
-        <v>93.9731</v>
+        <v>90.8989</v>
       </c>
       <c r="Y76" s="8" t="n">
-        <v>88.6315</v>
+        <v>83.3163</v>
       </c>
       <c r="Z76" s="8" t="n">
-        <v>93.7274</v>
+        <v>90.41900000000001</v>
       </c>
       <c r="AA76" s="9" t="n"/>
       <c r="AB76" s="9" t="n">
@@ -9307,22 +9299,1112 @@
       </c>
       <c r="AC76" s="5" t="inlineStr">
         <is>
+          <t>2:47:14.389924</t>
+        </is>
+      </c>
+      <c r="AD76" s="5" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1</t>
+        </is>
+      </c>
+      <c r="AE76" s="6" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1/S0/LEVIR/train_log.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="30" customHeight="1">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>SCTC-Run1</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>S0</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>S0_Clean_A2Net_LWGANet_L0</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="F77" s="6" t="inlineStr">
+        <is>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=none</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="H77" s="5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I77" s="5" t="n">
+        <v>2333</v>
+      </c>
+      <c r="J77" s="7" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="K77" s="5" t="inlineStr">
+        <is>
+          <t>poly</t>
+        </is>
+      </c>
+      <c r="L77" s="7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="M77" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N77" s="5" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="O77" s="7" t="n"/>
+      <c r="P77" s="7" t="n"/>
+      <c r="Q77" s="5" t="n"/>
+      <c r="R77" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="S77" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="T77" s="8" t="n">
+        <v>2.7676</v>
+      </c>
+      <c r="U77" s="8" t="n">
+        <v>81.14139999999999</v>
+      </c>
+      <c r="V77" s="8" t="n">
+        <v>84.9704</v>
+      </c>
+      <c r="W77" s="8" t="n">
+        <v>92.1679</v>
+      </c>
+      <c r="X77" s="8" t="n">
+        <v>83.01180000000001</v>
+      </c>
+      <c r="Y77" s="8" t="n">
+        <v>70.9573</v>
+      </c>
+      <c r="Z77" s="8" t="n">
+        <v>77.92609999999999</v>
+      </c>
+      <c r="AA77" s="9" t="n"/>
+      <c r="AB77" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC77" s="5" t="inlineStr">
+        <is>
+          <t>2:20:47.929272</t>
+        </is>
+      </c>
+      <c r="AD77" s="5" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1</t>
+        </is>
+      </c>
+      <c r="AE77" s="6" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1/S0/SYSU/train_log.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="30" customHeight="1">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>SCTC-Run1</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>S0</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>S0_Clean_A2Net_LWGANet_L0</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="F78" s="6" t="inlineStr">
+        <is>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=none</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="H78" s="5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I78" s="5" t="n">
+        <v>2333</v>
+      </c>
+      <c r="J78" s="7" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="K78" s="5" t="inlineStr">
+        <is>
+          <t>poly</t>
+        </is>
+      </c>
+      <c r="L78" s="7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="M78" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N78" s="5" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="O78" s="7" t="n"/>
+      <c r="P78" s="7" t="n"/>
+      <c r="Q78" s="5" t="n"/>
+      <c r="R78" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="S78" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="T78" s="8" t="n">
+        <v>2.7676</v>
+      </c>
+      <c r="U78" s="8" t="n">
+        <v>91.9434</v>
+      </c>
+      <c r="V78" s="8" t="n">
+        <v>95.20650000000001</v>
+      </c>
+      <c r="W78" s="8" t="n">
+        <v>99.4967</v>
+      </c>
+      <c r="X78" s="8" t="n">
+        <v>93.54649999999999</v>
+      </c>
+      <c r="Y78" s="8" t="n">
+        <v>87.87549999999999</v>
+      </c>
+      <c r="Z78" s="8" t="n">
+        <v>93.2847</v>
+      </c>
+      <c r="AA78" s="9" t="n"/>
+      <c r="AB78" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC78" s="5" t="inlineStr">
+        <is>
+          <t>2:43:01.630317</t>
+        </is>
+      </c>
+      <c r="AD78" s="5" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1</t>
+        </is>
+      </c>
+      <c r="AE78" s="6" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1/S0/WHU/train_log.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="30" customHeight="1">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>SCTC-Run1</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>S1_FullPixel_Symmetric_Calibration</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>CDD-CD-256</t>
+        </is>
+      </c>
+      <c r="F79" s="6" t="inlineStr">
+        <is>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=symmetric</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="H79" s="5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I79" s="5" t="n">
+        <v>2333</v>
+      </c>
+      <c r="J79" s="7" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="K79" s="5" t="inlineStr">
+        <is>
+          <t>poly</t>
+        </is>
+      </c>
+      <c r="L79" s="7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="M79" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N79" s="5" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="O79" s="7" t="n"/>
+      <c r="P79" s="7" t="n"/>
+      <c r="Q79" s="5" t="n"/>
+      <c r="R79" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="S79" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="T79" s="8" t="n">
+        <v>2.7676</v>
+      </c>
+      <c r="U79" s="8" t="n">
+        <v>97.39619999999999</v>
+      </c>
+      <c r="V79" s="8" t="n">
+        <v>97.7011</v>
+      </c>
+      <c r="W79" s="8" t="n">
+        <v>99.39570000000001</v>
+      </c>
+      <c r="X79" s="8" t="n">
+        <v>97.5484</v>
+      </c>
+      <c r="Y79" s="8" t="n">
+        <v>95.21420000000001</v>
+      </c>
+      <c r="Z79" s="8" t="n">
+        <v>97.2038</v>
+      </c>
+      <c r="AA79" s="9" t="n"/>
+      <c r="AB79" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC79" s="5" t="inlineStr">
+        <is>
+          <t>3:19:01.505607</t>
+        </is>
+      </c>
+      <c r="AD79" s="5" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1</t>
+        </is>
+      </c>
+      <c r="AE79" s="6" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1/S1/CDD/train_log.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="30" customHeight="1">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>SCTC-Run1</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>S1_FullPixel_Symmetric_Calibration</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="F80" s="6" t="inlineStr">
+        <is>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=symmetric</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="H80" s="5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I80" s="5" t="n">
+        <v>2333</v>
+      </c>
+      <c r="J80" s="7" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="K80" s="5" t="inlineStr">
+        <is>
+          <t>poly</t>
+        </is>
+      </c>
+      <c r="L80" s="7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="M80" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N80" s="5" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="O80" s="7" t="n"/>
+      <c r="P80" s="7" t="n"/>
+      <c r="Q80" s="5" t="n"/>
+      <c r="R80" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="S80" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="T80" s="8" t="n">
+        <v>2.7676</v>
+      </c>
+      <c r="U80" s="8" t="n">
+        <v>89.7944</v>
+      </c>
+      <c r="V80" s="8" t="n">
+        <v>92.1617</v>
+      </c>
+      <c r="W80" s="8" t="n">
+        <v>99.0911</v>
+      </c>
+      <c r="X80" s="8" t="n">
+        <v>90.96260000000001</v>
+      </c>
+      <c r="Y80" s="8" t="n">
+        <v>83.4233</v>
+      </c>
+      <c r="Z80" s="8" t="n">
+        <v>90.4842</v>
+      </c>
+      <c r="AA80" s="9" t="n"/>
+      <c r="AB80" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC80" s="5" t="inlineStr">
+        <is>
+          <t>0:33:15.349976</t>
+        </is>
+      </c>
+      <c r="AD80" s="5" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1</t>
+        </is>
+      </c>
+      <c r="AE80" s="6" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1/S1/LEVIR/train_log.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="30" customHeight="1">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>SCTC-Run1</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>S1_FullPixel_Symmetric_Calibration</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="inlineStr">
+        <is>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=symmetric</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="H81" s="5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I81" s="5" t="n">
+        <v>2333</v>
+      </c>
+      <c r="J81" s="7" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="K81" s="5" t="inlineStr">
+        <is>
+          <t>poly</t>
+        </is>
+      </c>
+      <c r="L81" s="7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="M81" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N81" s="5" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="O81" s="7" t="n"/>
+      <c r="P81" s="7" t="n"/>
+      <c r="Q81" s="5" t="n"/>
+      <c r="R81" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="S81" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="T81" s="8" t="n">
+        <v>2.7676</v>
+      </c>
+      <c r="U81" s="8" t="n">
+        <v>80.42610000000001</v>
+      </c>
+      <c r="V81" s="8" t="n">
+        <v>85.6097</v>
+      </c>
+      <c r="W81" s="8" t="n">
+        <v>92.19580000000001</v>
+      </c>
+      <c r="X81" s="8" t="n">
+        <v>82.93700000000001</v>
+      </c>
+      <c r="Y81" s="8" t="n">
+        <v>70.8481</v>
+      </c>
+      <c r="Z81" s="8" t="n">
+        <v>77.8843</v>
+      </c>
+      <c r="AA81" s="9" t="n"/>
+      <c r="AB81" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC81" s="5" t="inlineStr">
+        <is>
+          <t>3:32:56.072083</t>
+        </is>
+      </c>
+      <c r="AD81" s="5" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1</t>
+        </is>
+      </c>
+      <c r="AE81" s="6" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1/S1/SYSU/train_log.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="30" customHeight="1">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>SCTC-Run1</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>S1_FullPixel_Symmetric_Calibration</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="F82" s="6" t="inlineStr">
+        <is>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=symmetric</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="H82" s="5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I82" s="5" t="n">
+        <v>2333</v>
+      </c>
+      <c r="J82" s="7" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="K82" s="5" t="inlineStr">
+        <is>
+          <t>poly</t>
+        </is>
+      </c>
+      <c r="L82" s="7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="M82" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N82" s="5" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="O82" s="7" t="n"/>
+      <c r="P82" s="7" t="n"/>
+      <c r="Q82" s="5" t="n"/>
+      <c r="R82" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="S82" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="T82" s="8" t="n">
+        <v>2.7676</v>
+      </c>
+      <c r="U82" s="8" t="n">
+        <v>92.1589</v>
+      </c>
+      <c r="V82" s="8" t="n">
+        <v>95.1091</v>
+      </c>
+      <c r="W82" s="8" t="n">
+        <v>99.5009</v>
+      </c>
+      <c r="X82" s="8" t="n">
+        <v>93.61070000000001</v>
+      </c>
+      <c r="Y82" s="8" t="n">
+        <v>87.9889</v>
+      </c>
+      <c r="Z82" s="8" t="n">
+        <v>93.3511</v>
+      </c>
+      <c r="AA82" s="9" t="n"/>
+      <c r="AB82" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC82" s="5" t="inlineStr">
+        <is>
+          <t>2:40:44.864364</t>
+        </is>
+      </c>
+      <c r="AD82" s="5" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1</t>
+        </is>
+      </c>
+      <c r="AE82" s="6" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1/S1/WHU/train_log.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="30" customHeight="1">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>SCTC-Run1</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>S2_SCTC_UnchangedAware_Symmetric_CrossTemporal_Calibration</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>CDD-CD-256</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="inlineStr">
+        <is>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=sctc</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="H83" s="5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I83" s="5" t="n">
+        <v>2333</v>
+      </c>
+      <c r="J83" s="7" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="K83" s="5" t="inlineStr">
+        <is>
+          <t>poly</t>
+        </is>
+      </c>
+      <c r="L83" s="7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="M83" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N83" s="5" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="O83" s="7" t="n"/>
+      <c r="P83" s="7" t="n"/>
+      <c r="Q83" s="5" t="n"/>
+      <c r="R83" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="S83" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="T83" s="8" t="n">
+        <v>2.7676</v>
+      </c>
+      <c r="U83" s="8" t="n">
+        <v>97.4438</v>
+      </c>
+      <c r="V83" s="8" t="n">
+        <v>97.71940000000001</v>
+      </c>
+      <c r="W83" s="8" t="n">
+        <v>99.4038</v>
+      </c>
+      <c r="X83" s="8" t="n">
+        <v>97.5814</v>
+      </c>
+      <c r="Y83" s="8" t="n">
+        <v>95.277</v>
+      </c>
+      <c r="Z83" s="8" t="n">
+        <v>97.2414</v>
+      </c>
+      <c r="AA83" s="9" t="n"/>
+      <c r="AB83" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC83" s="5" t="inlineStr">
+        <is>
+          <t>2:52:30.285254</t>
+        </is>
+      </c>
+      <c r="AD83" s="5" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1</t>
+        </is>
+      </c>
+      <c r="AE83" s="6" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1/S2/CDD/train_log.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="30" customHeight="1">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>SCTC-Run1</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>S2_SCTC_UnchangedAware_Symmetric_CrossTemporal_Calibration</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>LEVIR-CD-256</t>
+        </is>
+      </c>
+      <c r="F84" s="6" t="inlineStr">
+        <is>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=sctc</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="H84" s="5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I84" s="5" t="n">
+        <v>2333</v>
+      </c>
+      <c r="J84" s="7" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="K84" s="5" t="inlineStr">
+        <is>
+          <t>poly</t>
+        </is>
+      </c>
+      <c r="L84" s="7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="M84" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N84" s="5" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="O84" s="7" t="n"/>
+      <c r="P84" s="7" t="n"/>
+      <c r="Q84" s="5" t="n"/>
+      <c r="R84" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="S84" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="T84" s="8" t="n">
+        <v>2.7676</v>
+      </c>
+      <c r="U84" s="8" t="n">
+        <v>90.1421</v>
+      </c>
+      <c r="V84" s="8" t="n">
+        <v>91.4601</v>
+      </c>
+      <c r="W84" s="8" t="n">
+        <v>99.069</v>
+      </c>
+      <c r="X84" s="8" t="n">
+        <v>90.7963</v>
+      </c>
+      <c r="Y84" s="8" t="n">
+        <v>83.14399999999999</v>
+      </c>
+      <c r="Z84" s="8" t="n">
+        <v>90.3061</v>
+      </c>
+      <c r="AA84" s="9" t="n"/>
+      <c r="AB84" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC84" s="5" t="inlineStr">
+        <is>
+          <t>3:18:11.767618</t>
+        </is>
+      </c>
+      <c r="AD84" s="5" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1</t>
+        </is>
+      </c>
+      <c r="AE84" s="6" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1/S2/LEVIR/train_log.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="30" customHeight="1">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>SCTC-Run1</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>S2_SCTC_UnchangedAware_Symmetric_CrossTemporal_Calibration</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>SYSU-CD-256</t>
+        </is>
+      </c>
+      <c r="F85" s="6" t="inlineStr">
+        <is>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=sctc</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="H85" s="5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I85" s="5" t="n">
+        <v>2333</v>
+      </c>
+      <c r="J85" s="7" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="K85" s="5" t="inlineStr">
+        <is>
+          <t>poly</t>
+        </is>
+      </c>
+      <c r="L85" s="7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="M85" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N85" s="5" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="O85" s="7" t="n"/>
+      <c r="P85" s="7" t="n"/>
+      <c r="Q85" s="5" t="n"/>
+      <c r="R85" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="S85" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="T85" s="8" t="n">
+        <v>2.7676</v>
+      </c>
+      <c r="U85" s="8" t="n">
+        <v>81.00070000000001</v>
+      </c>
+      <c r="V85" s="8" t="n">
+        <v>84.595</v>
+      </c>
+      <c r="W85" s="8" t="n">
+        <v>92.04090000000001</v>
+      </c>
+      <c r="X85" s="8" t="n">
+        <v>82.75879999999999</v>
+      </c>
+      <c r="Y85" s="8" t="n">
+        <v>70.5885</v>
+      </c>
+      <c r="Z85" s="8" t="n">
+        <v>77.5882</v>
+      </c>
+      <c r="AA85" s="9" t="n"/>
+      <c r="AB85" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC85" s="5" t="inlineStr">
+        <is>
+          <t>4:06:34.060509</t>
+        </is>
+      </c>
+      <c r="AD85" s="5" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1</t>
+        </is>
+      </c>
+      <c r="AE85" s="6" t="inlineStr">
+        <is>
+          <t>outputs/SCTC/Run1/S2/SYSU/train_log.txt</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="30" customHeight="1">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>SCTC-Run1</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>Full</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>S2_SCTC_UnchangedAware_Symmetric_CrossTemporal_Calibration</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>WHU-CD-256</t>
+        </is>
+      </c>
+      <c r="F86" s="6" t="inlineStr">
+        <is>
+          <t>batch=64; steps=40000; seed=2333; lr=0.0005; lr_mode=poly; wd=0.0001; backbone_lr=1.0; dice=batch; temporal=sctc</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="n">
+        <v>64</v>
+      </c>
+      <c r="H86" s="5" t="n">
+        <v>40000</v>
+      </c>
+      <c r="I86" s="5" t="n">
+        <v>2333</v>
+      </c>
+      <c r="J86" s="7" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="K86" s="5" t="inlineStr">
+        <is>
+          <t>poly</t>
+        </is>
+      </c>
+      <c r="L86" s="7" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="M86" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N86" s="5" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="O86" s="7" t="n"/>
+      <c r="P86" s="7" t="n"/>
+      <c r="Q86" s="5" t="n"/>
+      <c r="R86" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="S86" s="8" t="n">
+        <v>2.9131</v>
+      </c>
+      <c r="T86" s="8" t="n">
+        <v>2.7676</v>
+      </c>
+      <c r="U86" s="8" t="n">
+        <v>92.7942</v>
+      </c>
+      <c r="V86" s="8" t="n">
+        <v>95.1825</v>
+      </c>
+      <c r="W86" s="8" t="n">
+        <v>99.5278</v>
+      </c>
+      <c r="X86" s="8" t="n">
+        <v>93.9731</v>
+      </c>
+      <c r="Y86" s="8" t="n">
+        <v>88.6315</v>
+      </c>
+      <c r="Z86" s="8" t="n">
+        <v>93.7274</v>
+      </c>
+      <c r="AA86" s="9" t="n"/>
+      <c r="AB86" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC86" s="5" t="inlineStr">
+        <is>
           <t>2:08:54.218613</t>
         </is>
       </c>
-      <c r="AD76" s="5" t="inlineStr">
+      <c r="AD86" s="5" t="inlineStr">
         <is>
           <t>outputs/SCTC/Run1</t>
         </is>
       </c>
-      <c r="AE76" s="6" t="inlineStr">
+      <c r="AE86" s="6" t="inlineStr">
         <is>
           <t>outputs/SCTC/Run1/S2/WHU/train_log.txt</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="X2:X76">
+  <conditionalFormatting sqref="X2:X86">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -9347,7 +10429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -10647,6 +11729,176 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2</t>
+        </is>
+      </c>
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2/R0/SYSU/train_log.txt</t>
+        </is>
+      </c>
+      <c r="C77" s="11" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2</t>
+        </is>
+      </c>
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2/R0/WHU/train_log.txt</t>
+        </is>
+      </c>
+      <c r="C78" s="11" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2</t>
+        </is>
+      </c>
+      <c r="B79" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2/R1/SYSU/train_log.txt</t>
+        </is>
+      </c>
+      <c r="C79" s="11" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2</t>
+        </is>
+      </c>
+      <c r="B80" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2/R1/WHU/train_log.txt</t>
+        </is>
+      </c>
+      <c r="C80" s="11" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2</t>
+        </is>
+      </c>
+      <c r="B81" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2/R2/SYSU/train_log.txt</t>
+        </is>
+      </c>
+      <c r="C81" s="11" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2</t>
+        </is>
+      </c>
+      <c r="B82" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2/R2/WHU/train_log.txt</t>
+        </is>
+      </c>
+      <c r="C82" s="11" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2</t>
+        </is>
+      </c>
+      <c r="B83" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2/R3/SYSU/train_log.txt</t>
+        </is>
+      </c>
+      <c r="C83" s="11" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2</t>
+        </is>
+      </c>
+      <c r="B84" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2/R3/WHU/train_log.txt</t>
+        </is>
+      </c>
+      <c r="C84" s="11" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2</t>
+        </is>
+      </c>
+      <c r="B85" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2/R4/SYSU/train_log.txt</t>
+        </is>
+      </c>
+      <c r="C85" s="11" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2</t>
+        </is>
+      </c>
+      <c r="B86" s="11" t="inlineStr">
+        <is>
+          <t>outputs/SAGE-CD/Run2/R4/WHU/train_log.txt</t>
+        </is>
+      </c>
+      <c r="C86" s="11" t="inlineStr">
+        <is>
+          <t>complete</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>